<commit_message>
ignore chunkformer model and update crawler/tts code
</commit_message>
<xml_diff>
--- a/Craw_data/Begin.xlsx
+++ b/Craw_data/Begin.xlsx
@@ -8,24 +8,35 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CO_2026\TTS-DATA\Craw_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2499C054-F48C-4774-9692-4EA61C7B3B7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{296D9965-274B-4625-B3C2-1443DE9D51F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="18180" yWindow="0" windowWidth="7510" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5170" yWindow="2200" windowWidth="19200" windowHeight="11170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="28">
   <si>
     <t>https://www.youtube.com/@visaothenhipodcast</t>
   </si>
@@ -73,6 +84,42 @@
   </si>
   <si>
     <t>http://youtube.com/@ĐầuXanhMỏHỗn</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/@TNVlogs-Giaimalichsu</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/@heu.56mm</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/@thanhphohuetv</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/@podcast25phut33</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/@bhttv</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/@HieuTheConsul_Official</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/@thepodcastofthuan</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/@canthobaoptth</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/@baovaptthquangtri</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/@angiang24gio</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/@BáovàPTTHLâmĐồng1</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/@TruyềnhìnhQuảngNgãi</t>
   </si>
 </sst>
 </file>
@@ -401,7 +448,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A16"/>
+  <dimension ref="A1:A29"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="83.36328125" customWidth="1"/>
@@ -485,6 +532,71 @@
     <row r="16" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>14</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A17" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A18" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A19" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A20" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A21" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A22" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A23" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A24" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A25" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A26" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A27" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A28" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A29" s="1" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -505,6 +617,18 @@
     <hyperlink ref="A14" r:id="rId14" xr:uid="{123602B2-D16F-4607-95C0-60841D8CC928}"/>
     <hyperlink ref="A15" r:id="rId15" xr:uid="{F83E6CCD-3F05-422D-AB9A-B92A4086E445}"/>
     <hyperlink ref="A16" r:id="rId16" xr:uid="{3EF6AB45-03B1-4D2D-BB61-AB93597A69C4}"/>
+    <hyperlink ref="A17" r:id="rId17" xr:uid="{C57C7DC6-FEBC-4DAF-AE40-F9416F1BE453}"/>
+    <hyperlink ref="A18" r:id="rId18" xr:uid="{733AFE20-D1EA-45E1-8962-2D024E4F541A}"/>
+    <hyperlink ref="A19" r:id="rId19" xr:uid="{8B4FA3A5-9235-4B76-9B96-B574DDCEA069}"/>
+    <hyperlink ref="A20" r:id="rId20" xr:uid="{3AF65C88-0FEB-4CD9-B887-92B72E304198}"/>
+    <hyperlink ref="A21" r:id="rId21" xr:uid="{E05AFFEB-EB6D-4EF4-AB88-259A826D5D04}"/>
+    <hyperlink ref="A23" r:id="rId22" xr:uid="{7F4E223C-0E2A-4E80-9AA0-97137C6ABDB9}"/>
+    <hyperlink ref="A25" r:id="rId23" xr:uid="{B36DEDEA-6990-40A7-B841-74437651CDEF}"/>
+    <hyperlink ref="A26" r:id="rId24" xr:uid="{8C37309C-E23D-43DC-8EAE-129109712FBB}"/>
+    <hyperlink ref="A27" r:id="rId25" xr:uid="{1F2D6E84-8F50-4BE8-9EC1-73FA46D2441C}"/>
+    <hyperlink ref="A28" r:id="rId26" xr:uid="{D149AF92-9D10-4603-A14A-11D35C33B309}"/>
+    <hyperlink ref="A29" r:id="rId27" xr:uid="{B9B4140A-DB21-473C-8C4C-64CDD58C5494}"/>
+    <hyperlink ref="A24" r:id="rId28" xr:uid="{782DE413-FBDD-403E-9077-A79DF7960C82}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update code to support multi-threading and fix orphaned files logic
</commit_message>
<xml_diff>
--- a/Craw_data/Begin.xlsx
+++ b/Craw_data/Begin.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CO_2026\TTS-DATA\Craw_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{296D9965-274B-4625-B3C2-1443DE9D51F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{724748BB-4DF2-49FF-A718-12550B1F4FF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5170" yWindow="2200" windowWidth="19200" windowHeight="11170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="35">
   <si>
     <t>https://www.youtube.com/@visaothenhipodcast</t>
   </si>
@@ -120,6 +120,27 @@
   </si>
   <si>
     <t>https://www.youtube.com/@TruyềnhìnhQuảngNgãi</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/@TuanTienTi2911</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/@MèoGiảiThích</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/@vtv24</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/@vietnamplus-w3i</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/@hoainiem-kinhhong</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/@TruyenDem-QStudio</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/@kenhCoVan</t>
   </si>
 </sst>
 </file>
@@ -448,155 +469,195 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A29"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:A37"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="83.36328125" customWidth="1"/>
+    <col min="1" max="1" width="83.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>27</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A30" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A31" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A32" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A33" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A34" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A35" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A36" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A37" s="1" t="s">
+        <v>34</v>
       </c>
     </row>
   </sheetData>
@@ -629,6 +690,14 @@
     <hyperlink ref="A28" r:id="rId26" xr:uid="{D149AF92-9D10-4603-A14A-11D35C33B309}"/>
     <hyperlink ref="A29" r:id="rId27" xr:uid="{B9B4140A-DB21-473C-8C4C-64CDD58C5494}"/>
     <hyperlink ref="A24" r:id="rId28" xr:uid="{782DE413-FBDD-403E-9077-A79DF7960C82}"/>
+    <hyperlink ref="A30" r:id="rId29" xr:uid="{3A8BED86-E952-4619-BC0D-949FFC83D34F}"/>
+    <hyperlink ref="A31" r:id="rId30" xr:uid="{A72EC037-894E-4499-915A-21833C8B475D}"/>
+    <hyperlink ref="A32" r:id="rId31" xr:uid="{84145EB4-503A-4BBC-B5F4-AA12680F1B42}"/>
+    <hyperlink ref="A33" r:id="rId32" xr:uid="{78503CFD-A210-40A1-A32E-1DBF69954FCC}"/>
+    <hyperlink ref="A34" r:id="rId33" xr:uid="{FBEC8A15-FAE7-41D1-A06C-8A19AA6A25F8}"/>
+    <hyperlink ref="A35" r:id="rId34" xr:uid="{E30B944D-C752-4425-BC84-E4665C486326}"/>
+    <hyperlink ref="A36" r:id="rId35" xr:uid="{4A24A352-8F1D-468C-9E40-C69DBA6AB5DA}"/>
+    <hyperlink ref="A37" r:id="rId36" xr:uid="{F66A2622-86CD-4881-AFEA-96E34DE2E522}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>